<commit_message>
Killable Buildings/Units for Joan
</commit_message>
<xml_diff>
--- a/docs/Logic Requirements/Ageipelago Attila the Hun.xlsx
+++ b/docs/Logic Requirements/Ageipelago Attila the Hun.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\stefb\OneDrive\Desktop\Logic Requirements\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73F383AC-5211-4BBA-B610-7265FE959CE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6984C88F-F72A-45E1-B416-A20AE792BBE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="639" activeTab="5" xr2:uid="{B80992DC-780F-4856-A6B0-D26FA95FCBC0}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="639" activeTab="6" xr2:uid="{B80992DC-780F-4856-A6B0-D26FA95FCBC0}"/>
   </bookViews>
   <sheets>
     <sheet name="Attila the Hun" sheetId="1" r:id="rId1"/>
@@ -4653,20 +4653,6 @@
   </si>
   <si>
     <r>
-      <t xml:space="preserve">Spearman
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>(not on Hard)</t>
-    </r>
-  </si>
-  <si>
-    <r>
       <rPr>
         <sz val="14"/>
         <color rgb="FF0070C0"/>
@@ -4771,10 +4757,6 @@
   </si>
   <si>
     <t>Crossbowman</t>
-  </si>
-  <si>
-    <t>Pikeman
-(not on Standard)</t>
   </si>
   <si>
     <t>Trade Cart</t>
@@ -5154,21 +5136,6 @@
   </si>
   <si>
     <r>
-      <t xml:space="preserve">Two-Handed Swordsman
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>(not on Standard)</t>
-    </r>
-  </si>
-  <si>
-    <r>
       <t xml:space="preserve">Champion
 </t>
     </r>
@@ -5184,21 +5151,6 @@
   </si>
   <si>
     <r>
-      <t xml:space="preserve">Elite Huskarl
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>(not on Standard)</t>
-    </r>
-  </si>
-  <si>
-    <r>
       <t xml:space="preserve">Capped Ram
 </t>
     </r>
@@ -5303,6 +5255,112 @@
   </si>
   <si>
     <t>Aqueduct</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Pikeman
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>(not on Standard)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="14"/>
+        <color rgb="FF2FE2F5"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Spearman</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FF2FE2F5"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>(not on Hard)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="14"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Elite Huskarl</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>(not on Standard)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="14"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Two-Handed Swordsman</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>(not on Standard)</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -5711,7 +5769,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -5825,9 +5883,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="32" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -6443,13 +6498,13 @@
         <v>74</v>
       </c>
       <c r="K8" s="7" t="s">
+        <v>278</v>
+      </c>
+      <c r="L8" s="7" t="s">
+        <v>279</v>
+      </c>
+      <c r="M8" s="7" t="s">
         <v>280</v>
-      </c>
-      <c r="L8" s="7" t="s">
-        <v>281</v>
-      </c>
-      <c r="M8" s="7" t="s">
-        <v>282</v>
       </c>
       <c r="N8" s="7" t="s">
         <v>73</v>
@@ -6559,7 +6614,7 @@
       <c r="H3" s="8" t="s">
         <v>112</v>
       </c>
-      <c r="K3" s="18" t="s">
+      <c r="K3" s="17" t="s">
         <v>212</v>
       </c>
       <c r="L3" s="8" t="s">
@@ -6622,7 +6677,7 @@
       <c r="D6" s="8" t="s">
         <v>112</v>
       </c>
-      <c r="G6" s="16" t="s">
+      <c r="G6" s="9" t="s">
         <v>189</v>
       </c>
       <c r="H6" s="8" t="s">
@@ -6645,7 +6700,7 @@
       <c r="D7" s="8" t="s">
         <v>112</v>
       </c>
-      <c r="G7" s="9" t="s">
+      <c r="G7" s="16" t="s">
         <v>190</v>
       </c>
       <c r="H7" s="8" t="s">
@@ -6927,7 +6982,7 @@
       <c r="H19" s="8" t="s">
         <v>165</v>
       </c>
-      <c r="K19" s="22" t="s">
+      <c r="K19" s="20" t="s">
         <v>227</v>
       </c>
       <c r="L19" s="8" t="s">
@@ -6997,7 +7052,7 @@
         <v>207</v>
       </c>
       <c r="K22" s="20" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="L22" s="8" t="s">
         <v>165</v>
@@ -7252,7 +7307,7 @@
         <v>112</v>
       </c>
       <c r="G8" s="26" t="s">
-        <v>238</v>
+        <v>304</v>
       </c>
       <c r="H8" s="8" t="s">
         <v>112</v>
@@ -7275,13 +7330,13 @@
         <v>112</v>
       </c>
       <c r="G9" s="26" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="H9" s="8" t="s">
         <v>112</v>
       </c>
       <c r="K9" s="22" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="L9" s="8" t="s">
         <v>112</v>
@@ -7303,7 +7358,7 @@
       <c r="H10" s="8" t="s">
         <v>112</v>
       </c>
-      <c r="K10" s="30" t="s">
+      <c r="K10" s="28" t="s">
         <v>227</v>
       </c>
       <c r="L10" s="8" t="s">
@@ -7407,7 +7462,7 @@
         <v>182</v>
       </c>
       <c r="G15" s="9" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="H15" s="5" t="s">
         <v>181</v>
@@ -7430,7 +7485,7 @@
         <v>112</v>
       </c>
       <c r="G16" s="9" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="H16" s="5" t="s">
         <v>181</v>
@@ -7453,7 +7508,7 @@
         <v>112</v>
       </c>
       <c r="G17" s="9" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="H17" s="5" t="s">
         <v>181</v>
@@ -7476,7 +7531,7 @@
         <v>112</v>
       </c>
       <c r="G18" s="19" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="H18" s="5" t="s">
         <v>181</v>
@@ -7507,7 +7562,7 @@
         <v>208</v>
       </c>
       <c r="H20" s="5" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="K20" s="27" t="s">
         <v>225</v>
@@ -7544,8 +7599,8 @@
       </c>
     </row>
     <row r="24" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="K24" s="18" t="s">
-        <v>246</v>
+      <c r="K24" s="17" t="s">
+        <v>245</v>
       </c>
       <c r="L24" s="8" t="s">
         <v>112</v>
@@ -7553,7 +7608,7 @@
     </row>
     <row r="25" spans="2:12" ht="112.5" x14ac:dyDescent="0.25">
       <c r="K25" s="19" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="L25" s="5" t="s">
         <v>181</v>
@@ -7637,7 +7692,7 @@
         <v>112</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="H4" s="8" t="s">
         <v>112</v>
@@ -7660,7 +7715,7 @@
         <v>112</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="H5" s="8" t="s">
         <v>112</v>
@@ -7706,7 +7761,7 @@
         <v>112</v>
       </c>
       <c r="G7" s="20" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="H7" s="8" t="s">
         <v>112</v>
@@ -7734,8 +7789,8 @@
       <c r="H8" s="8" t="s">
         <v>112</v>
       </c>
-      <c r="K8" s="23" t="s">
-        <v>246</v>
+      <c r="K8" s="21" t="s">
+        <v>245</v>
       </c>
       <c r="L8" s="8" t="s">
         <v>112</v>
@@ -7798,7 +7853,7 @@
         <v>112</v>
       </c>
       <c r="G11" s="21" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="H11" s="8" t="s">
         <v>112</v>
@@ -7821,7 +7876,7 @@
         <v>112</v>
       </c>
       <c r="G12" s="21" t="s">
-        <v>252</v>
+        <v>303</v>
       </c>
       <c r="H12" s="8" t="s">
         <v>112</v>
@@ -7844,7 +7899,7 @@
         <v>167</v>
       </c>
       <c r="G13" s="23" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="H13" s="8" t="s">
         <v>112</v>
@@ -7916,7 +7971,7 @@
         <v>208</v>
       </c>
       <c r="H16" s="8" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="K16" s="20" t="s">
         <v>218</v>
@@ -7936,10 +7991,10 @@
         <v>170</v>
       </c>
       <c r="G17" s="22" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="H17" s="8" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="K17" s="20" t="s">
         <v>223</v>
@@ -7959,10 +8014,10 @@
         <v>112</v>
       </c>
       <c r="G18" s="31" t="s">
+        <v>253</v>
+      </c>
+      <c r="H18" s="8" t="s">
         <v>255</v>
-      </c>
-      <c r="H18" s="8" t="s">
-        <v>257</v>
       </c>
       <c r="K18" s="20" t="s">
         <v>224</v>
@@ -7982,7 +8037,7 @@
         <v>112</v>
       </c>
       <c r="G19" s="31" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="H19" s="8" t="s">
         <v>112</v>
@@ -8005,7 +8060,7 @@
         <v>170</v>
       </c>
       <c r="K20" s="19" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="L20" s="8" t="s">
         <v>112</v>
@@ -8022,7 +8077,7 @@
         <v>112</v>
       </c>
       <c r="K21" s="19" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="L21" s="8" t="s">
         <v>112</v>
@@ -8030,7 +8085,7 @@
     </row>
     <row r="22" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
       <c r="K22" s="19" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="L22" s="8" t="s">
         <v>112</v>
@@ -8062,23 +8117,23 @@
     </row>
     <row r="26" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
       <c r="K26" s="19" t="s">
+        <v>259</v>
+      </c>
+      <c r="L26" s="8" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="27" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="K27" s="19" t="s">
+        <v>260</v>
+      </c>
+      <c r="L27" s="8" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="28" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="K28" s="19" t="s">
         <v>261</v>
-      </c>
-      <c r="L26" s="8" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="27" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="K27" s="31" t="s">
-        <v>262</v>
-      </c>
-      <c r="L27" s="8" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="28" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="K28" s="31" t="s">
-        <v>263</v>
       </c>
       <c r="L28" s="8" t="s">
         <v>112</v>
@@ -8209,7 +8264,7 @@
         <v>177</v>
       </c>
       <c r="G6" s="9" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="H6" s="8" t="s">
         <v>112</v>
@@ -8255,10 +8310,10 @@
         <v>176</v>
       </c>
       <c r="G8" s="17" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="H8" s="8" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="K8" s="17" t="s">
         <v>214</v>
@@ -8278,10 +8333,10 @@
         <v>171</v>
       </c>
       <c r="G9" s="17" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="H9" s="8" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="K9" s="17" t="s">
         <v>233</v>
@@ -8301,10 +8356,10 @@
         <v>112</v>
       </c>
       <c r="G10" s="17" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="H10" s="8" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="K10" s="17" t="s">
         <v>216</v>
@@ -8315,10 +8370,10 @@
     </row>
     <row r="11" spans="2:12" ht="37.5" x14ac:dyDescent="0.25">
       <c r="G11" s="26" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="H11" s="8" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="K11" s="17" t="s">
         <v>217</v>
@@ -8329,10 +8384,10 @@
     </row>
     <row r="12" spans="2:12" ht="37.5" x14ac:dyDescent="0.25">
       <c r="G12" s="26" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="H12" s="8" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="K12" s="17" t="s">
         <v>220</v>
@@ -8346,10 +8401,10 @@
         <v>203</v>
       </c>
       <c r="H13" s="8" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="K13" s="17" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="L13" s="8" t="s">
         <v>112</v>
@@ -8357,10 +8412,10 @@
     </row>
     <row r="14" spans="2:12" ht="37.5" x14ac:dyDescent="0.25">
       <c r="G14" s="26" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="H14" s="8" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="K14" s="17" t="s">
         <v>230</v>
@@ -8371,10 +8426,10 @@
     </row>
     <row r="15" spans="2:12" ht="37.5" x14ac:dyDescent="0.25">
       <c r="G15" s="26" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="H15" s="8" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="K15" s="21" t="s">
         <v>223</v>
@@ -8385,10 +8440,10 @@
     </row>
     <row r="16" spans="2:12" ht="37.5" x14ac:dyDescent="0.25">
       <c r="G16" s="26" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="H16" s="8" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="K16" s="21" t="s">
         <v>218</v>
@@ -8399,10 +8454,10 @@
     </row>
     <row r="17" spans="7:14" ht="37.5" x14ac:dyDescent="0.25">
       <c r="G17" s="26" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="H17" s="8" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="K17" s="21" t="s">
         <v>228</v>
@@ -8416,7 +8471,7 @@
         <v>235</v>
       </c>
       <c r="H18" s="8" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="K18" s="26" t="s">
         <v>213</v>
@@ -8427,10 +8482,10 @@
     </row>
     <row r="19" spans="7:14" ht="37.5" x14ac:dyDescent="0.25">
       <c r="G19" s="26" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="H19" s="8" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="K19" s="26" t="s">
         <v>231</v>
@@ -8441,13 +8496,13 @@
     </row>
     <row r="20" spans="7:14" ht="37.5" x14ac:dyDescent="0.25">
       <c r="G20" s="26" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="H20" s="8" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="K20" s="26" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="L20" s="8" t="s">
         <v>112</v>
@@ -8455,13 +8510,13 @@
     </row>
     <row r="21" spans="7:14" ht="37.5" x14ac:dyDescent="0.25">
       <c r="G21" s="26" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="H21" s="8" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="K21" s="26" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="L21" s="8" t="s">
         <v>112</v>
@@ -8469,13 +8524,13 @@
     </row>
     <row r="22" spans="7:14" ht="37.5" x14ac:dyDescent="0.25">
       <c r="G22" s="26" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="H22" s="8" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="K22" s="35" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="L22" s="32" t="s">
         <v>112</v>
@@ -8483,53 +8538,53 @@
     </row>
     <row r="23" spans="7:14" ht="37.5" x14ac:dyDescent="0.25">
       <c r="G23" s="19" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="H23" s="8" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="K23" s="33"/>
       <c r="L23" s="33"/>
     </row>
     <row r="24" spans="7:14" ht="37.5" x14ac:dyDescent="0.25">
       <c r="G24" s="24" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="H24" s="32" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="K24" s="25"/>
       <c r="L24" s="25"/>
     </row>
     <row r="25" spans="7:14" ht="37.5" x14ac:dyDescent="0.25">
       <c r="G25" s="21" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="H25" s="8" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="K25" s="25"/>
       <c r="L25" s="25"/>
       <c r="N25" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="26" spans="7:14" ht="37.5" x14ac:dyDescent="0.25">
       <c r="G26" s="21" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="H26" s="8" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="K26" s="25"/>
       <c r="L26" s="25"/>
     </row>
     <row r="27" spans="7:14" ht="37.5" x14ac:dyDescent="0.25">
       <c r="G27" s="21" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="H27" s="8" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="K27" s="25"/>
       <c r="L27" s="25"/>
@@ -8618,7 +8673,7 @@
         <v>177</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="H4" s="8" t="s">
         <v>112</v>
@@ -8670,7 +8725,7 @@
         <v>112</v>
       </c>
       <c r="K6" s="27" t="s">
-        <v>294</v>
+        <v>290</v>
       </c>
       <c r="L6" s="8" t="s">
         <v>112</v>
@@ -8710,7 +8765,7 @@
         <v>112</v>
       </c>
       <c r="G8" s="27" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="H8" s="8" t="s">
         <v>112</v>
@@ -8730,7 +8785,7 @@
         <v>112</v>
       </c>
       <c r="K9" s="38" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="L9" s="8" t="s">
         <v>112</v>
@@ -8752,7 +8807,7 @@
     </row>
     <row r="11" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
       <c r="G11" s="20" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="H11" s="8" t="s">
         <v>112</v>
@@ -8766,7 +8821,7 @@
     </row>
     <row r="12" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
       <c r="G12" s="20" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="H12" s="8" t="s">
         <v>112</v>
@@ -8780,13 +8835,13 @@
     </row>
     <row r="13" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
       <c r="G13" s="22" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="H13" s="8" t="s">
         <v>112</v>
       </c>
       <c r="K13" s="20" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="L13" s="8" t="s">
         <v>112</v>
@@ -8794,7 +8849,7 @@
     </row>
     <row r="14" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
       <c r="G14" s="20" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="H14" s="8" t="s">
         <v>112</v>
@@ -8808,7 +8863,7 @@
     </row>
     <row r="15" spans="2:12" ht="37.5" x14ac:dyDescent="0.25">
       <c r="G15" s="20" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="H15" s="8" t="s">
         <v>112</v>
@@ -8822,7 +8877,7 @@
     </row>
     <row r="16" spans="2:12" ht="56.25" x14ac:dyDescent="0.25">
       <c r="G16" s="20" t="s">
-        <v>285</v>
+        <v>306</v>
       </c>
       <c r="H16" s="8" t="s">
         <v>112</v>
@@ -8836,12 +8891,12 @@
     </row>
     <row r="17" spans="7:12" ht="37.5" x14ac:dyDescent="0.25">
       <c r="G17" s="20" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
       <c r="H17" s="8" t="s">
         <v>112</v>
       </c>
-      <c r="K17" s="39" t="s">
+      <c r="K17" s="26" t="s">
         <v>227</v>
       </c>
       <c r="L17" s="8" t="s">
@@ -8850,7 +8905,7 @@
     </row>
     <row r="18" spans="7:12" ht="37.5" x14ac:dyDescent="0.25">
       <c r="G18" s="20" t="s">
-        <v>287</v>
+        <v>305</v>
       </c>
       <c r="H18" s="8" t="s">
         <v>112</v>
@@ -8864,7 +8919,7 @@
     </row>
     <row r="19" spans="7:12" ht="37.5" x14ac:dyDescent="0.25">
       <c r="G19" s="20" t="s">
-        <v>288</v>
+        <v>284</v>
       </c>
       <c r="H19" s="8" t="s">
         <v>112</v>
@@ -8892,13 +8947,13 @@
     </row>
     <row r="21" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
       <c r="G21" s="26" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="H21" s="8" t="s">
         <v>112</v>
       </c>
-      <c r="K21" s="40" t="s">
-        <v>295</v>
+      <c r="K21" s="39" t="s">
+        <v>291</v>
       </c>
       <c r="L21" s="32" t="s">
         <v>112</v>
@@ -8906,7 +8961,7 @@
     </row>
     <row r="22" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
       <c r="G22" s="35" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="H22" s="32" t="s">
         <v>112</v>
@@ -8926,7 +8981,7 @@
     </row>
     <row r="24" spans="7:12" ht="37.5" x14ac:dyDescent="0.25">
       <c r="G24" s="26" t="s">
-        <v>289</v>
+        <v>285</v>
       </c>
       <c r="H24" s="8" t="s">
         <v>112</v>
@@ -8936,7 +8991,7 @@
     </row>
     <row r="25" spans="7:12" ht="37.5" x14ac:dyDescent="0.25">
       <c r="G25" s="20" t="s">
-        <v>290</v>
+        <v>286</v>
       </c>
       <c r="H25" s="8" t="s">
         <v>112</v>
@@ -8955,8 +9010,8 @@
       <c r="L26" s="25"/>
     </row>
     <row r="27" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="G27" s="19" t="s">
-        <v>291</v>
+      <c r="G27" s="31" t="s">
+        <v>287</v>
       </c>
       <c r="H27" s="8" t="s">
         <v>112</v>
@@ -8966,7 +9021,7 @@
     </row>
     <row r="28" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
       <c r="G28" s="19" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="H28" s="8" t="s">
         <v>112</v>
@@ -8976,7 +9031,7 @@
     </row>
     <row r="29" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
       <c r="G29" s="19" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="H29" s="8" t="s">
         <v>112</v>
@@ -8986,7 +9041,7 @@
     </row>
     <row r="30" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
       <c r="G30" s="19" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="H30" s="8" t="s">
         <v>112</v>
@@ -8996,7 +9051,7 @@
     </row>
     <row r="31" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
       <c r="G31" s="24" t="s">
-        <v>293</v>
+        <v>289</v>
       </c>
       <c r="H31" s="32" t="s">
         <v>112</v>
@@ -9130,8 +9185,8 @@
       <c r="H3" s="6" t="s">
         <v>112</v>
       </c>
-      <c r="K3" s="42" t="s">
-        <v>258</v>
+      <c r="K3" s="41" t="s">
+        <v>256</v>
       </c>
       <c r="L3" s="6" t="s">
         <v>112</v>
@@ -9154,7 +9209,7 @@
         <v>112</v>
       </c>
       <c r="K4" s="21" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="L4" s="9" t="s">
         <v>112</v>
@@ -9171,13 +9226,13 @@
         <v>178</v>
       </c>
       <c r="G5" s="9" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="H5" s="9" t="s">
         <v>112</v>
       </c>
       <c r="K5" s="21" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="L5" s="9" t="s">
         <v>112</v>
@@ -9194,13 +9249,13 @@
         <v>178</v>
       </c>
       <c r="G6" s="16" t="s">
-        <v>296</v>
+        <v>292</v>
       </c>
       <c r="H6" s="9" t="s">
         <v>112</v>
       </c>
-      <c r="K6" s="23" t="s">
-        <v>262</v>
+      <c r="K6" s="21" t="s">
+        <v>260</v>
       </c>
       <c r="L6" s="9" t="s">
         <v>112</v>
@@ -9222,8 +9277,8 @@
       <c r="H7" s="9" t="s">
         <v>112</v>
       </c>
-      <c r="K7" s="23" t="s">
-        <v>263</v>
+      <c r="K7" s="21" t="s">
+        <v>261</v>
       </c>
       <c r="L7" s="9" t="s">
         <v>112</v>
@@ -9263,7 +9318,7 @@
         <v>178</v>
       </c>
       <c r="G9" s="21" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="H9" s="9" t="s">
         <v>112</v>
@@ -9286,7 +9341,7 @@
         <v>178</v>
       </c>
       <c r="G10" s="21" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="H10" s="9" t="s">
         <v>112</v>
@@ -9332,13 +9387,13 @@
         <v>178</v>
       </c>
       <c r="G12" s="21" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="H12" s="9" t="s">
         <v>112</v>
       </c>
       <c r="K12" s="21" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="L12" s="9" t="s">
         <v>112</v>
@@ -9355,7 +9410,7 @@
         <v>178</v>
       </c>
       <c r="G13" s="23" t="s">
-        <v>297</v>
+        <v>293</v>
       </c>
       <c r="H13" s="9" t="s">
         <v>112</v>
@@ -9378,7 +9433,7 @@
         <v>178</v>
       </c>
       <c r="G14" s="21" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="H14" s="9" t="s">
         <v>112</v>
@@ -9401,7 +9456,7 @@
         <v>112</v>
       </c>
       <c r="G15" s="21" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="H15" s="9" t="s">
         <v>112</v>
@@ -9415,7 +9470,7 @@
     </row>
     <row r="16" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
       <c r="G16" s="20" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="H16" s="9" t="s">
         <v>112</v>
@@ -9443,7 +9498,7 @@
     </row>
     <row r="18" spans="7:12" ht="37.5" x14ac:dyDescent="0.25">
       <c r="G18" s="20" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="H18" s="9" t="s">
         <v>112</v>
@@ -9457,7 +9512,7 @@
     </row>
     <row r="19" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
       <c r="G19" s="20" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="H19" s="9" t="s">
         <v>112</v>
@@ -9471,13 +9526,13 @@
     </row>
     <row r="20" spans="7:12" ht="37.5" x14ac:dyDescent="0.25">
       <c r="G20" s="28" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="H20" s="9" t="s">
         <v>112</v>
       </c>
       <c r="K20" s="21" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="L20" s="9" t="s">
         <v>112</v>
@@ -9485,7 +9540,7 @@
     </row>
     <row r="21" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
       <c r="G21" s="18" t="s">
-        <v>299</v>
+        <v>295</v>
       </c>
       <c r="H21" s="9" t="s">
         <v>112</v>
@@ -9499,13 +9554,13 @@
     </row>
     <row r="22" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
       <c r="G22" s="17" t="s">
-        <v>293</v>
+        <v>289</v>
       </c>
       <c r="H22" s="9" t="s">
         <v>112</v>
       </c>
       <c r="K22" s="22" t="s">
-        <v>303</v>
+        <v>299</v>
       </c>
       <c r="L22" s="9" t="s">
         <v>112</v>
@@ -9527,7 +9582,7 @@
     </row>
     <row r="24" spans="7:12" ht="37.5" x14ac:dyDescent="0.25">
       <c r="G24" s="17" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="H24" s="9" t="s">
         <v>112</v>
@@ -9541,7 +9596,7 @@
     </row>
     <row r="25" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
       <c r="G25" s="19" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="H25" s="9" t="s">
         <v>112</v>
@@ -9555,13 +9610,13 @@
     </row>
     <row r="26" spans="7:12" ht="318.75" x14ac:dyDescent="0.25">
       <c r="G26" s="31" t="s">
-        <v>300</v>
+        <v>296</v>
       </c>
       <c r="H26" s="8" t="s">
         <v>178</v>
       </c>
       <c r="K26" s="31" t="s">
-        <v>304</v>
+        <v>300</v>
       </c>
       <c r="L26" s="9" t="s">
         <v>112</v>
@@ -9569,13 +9624,13 @@
     </row>
     <row r="27" spans="7:12" ht="37.5" x14ac:dyDescent="0.25">
       <c r="G27" s="21" t="s">
+        <v>297</v>
+      </c>
+      <c r="H27" s="9" t="s">
+        <v>255</v>
+      </c>
+      <c r="K27" s="31" t="s">
         <v>301</v>
-      </c>
-      <c r="H27" s="9" t="s">
-        <v>257</v>
-      </c>
-      <c r="K27" s="31" t="s">
-        <v>305</v>
       </c>
       <c r="L27" s="9" t="s">
         <v>112</v>
@@ -9583,24 +9638,24 @@
     </row>
     <row r="28" spans="7:12" ht="37.5" x14ac:dyDescent="0.25">
       <c r="G28" s="23" t="s">
+        <v>298</v>
+      </c>
+      <c r="H28" s="9" t="s">
+        <v>255</v>
+      </c>
+      <c r="K28" s="42" t="s">
         <v>302</v>
       </c>
-      <c r="H28" s="9" t="s">
-        <v>257</v>
-      </c>
-      <c r="K28" s="43" t="s">
-        <v>306</v>
-      </c>
       <c r="L28" s="36" t="s">
         <v>112</v>
       </c>
     </row>
     <row r="29" spans="7:12" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="G29" s="41" t="s">
+      <c r="G29" s="40" t="s">
+        <v>253</v>
+      </c>
+      <c r="H29" s="36" t="s">
         <v>255</v>
-      </c>
-      <c r="H29" s="36" t="s">
-        <v>257</v>
       </c>
       <c r="K29" s="33"/>
       <c r="L29" s="33"/>

</xml_diff>